<commit_message>
updated guide that data is not stored on server
</commit_message>
<xml_diff>
--- a/toy-data.xlsx
+++ b/toy-data.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robert.elder/Documents/experiments/09-ivivc-tool/app-v0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C88C4FA0-3C55-7E4B-A3B1-5497FC7DA80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5C678C-FBC5-0D40-86CD-5DF063807DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6520" yWindow="4900" windowWidth="28040" windowHeight="17440" xr2:uid="{B6545CCB-97A8-EF41-B081-88DEAE44E7A3}"/>
+    <workbookView xWindow="6520" yWindow="4900" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{B6545CCB-97A8-EF41-B081-88DEAE44E7A3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Stretched exponentials (smooth)" sheetId="1" r:id="rId1"/>
+    <sheet name="Stretched exponentials (noisy)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
   <si>
     <t>time1</t>
   </si>
@@ -830,4 +831,372 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCEB4C4-5FEF-AF4C-AD93-CE1A46E49E5E}">
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>0.90794182823391523</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>0.90916611307324613</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.9303926169796779</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>0.86110847602992424</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>0.90458646429633349</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>0.71690226945336</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.84914599976736727</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>0.60741956289562526</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.80686543723617921</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>0.50513721665221289</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.70033170322047955</v>
+      </c>
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>0.43495995465187792</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>0.61308983248281401</v>
+      </c>
+      <c r="C9">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>0.32838898943259243</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>0.50878072836002508</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>0.31043847773131578</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>0.46914199861615591</v>
+      </c>
+      <c r="C11">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0.25396627084167012</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0.31007252914657379</v>
+      </c>
+      <c r="C12">
+        <v>20</v>
+      </c>
+      <c r="D12">
+        <v>0.17468306146404089</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>0.30676595146124291</v>
+      </c>
+      <c r="C13">
+        <v>22</v>
+      </c>
+      <c r="D13">
+        <v>0.14501256722123951</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>0.2645273657660494</v>
+      </c>
+      <c r="C14">
+        <v>24</v>
+      </c>
+      <c r="D14">
+        <v>8.1894031562552483E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>0.15621647904113339</v>
+      </c>
+      <c r="C15">
+        <v>26</v>
+      </c>
+      <c r="D15">
+        <v>6.6826291772344906E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>0.15990764010477229</v>
+      </c>
+      <c r="C16">
+        <v>28</v>
+      </c>
+      <c r="D16">
+        <v>7.2584589963362992E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>0.1187261348440698</v>
+      </c>
+      <c r="C17">
+        <v>30</v>
+      </c>
+      <c r="D17">
+        <v>5.9051202255119291E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>9.5401894443902652E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>6.4291204191874396E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>5.6061223880019537E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>1.4301484609982439E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>2.55603920382385E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>2.2857500242050521E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>3.7892843986940483E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>2.472623433754579E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>1.8370047150848692E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>1.1728861503672319E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>1.5138979887977621E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>2.0061710738640319E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>